<commit_message>
Updated the fields to accept multiple ID instead of one Type(DOI)
</commit_message>
<xml_diff>
--- a/raid-agency-app/public/templates/related-objects-template.xlsx
+++ b/raid-agency-app/public/templates/related-objects-template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\raid-au\raid-agency-app\public\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\raid-au\raid-agency-app\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09B3170E-A12D-4FD6-9C27-FD56F0FFA3CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11C8B814-CB0D-4777-AE8D-22F7C30BDEBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="2205" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,9 +32,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
   <si>
-    <t>DOI URL</t>
-  </si>
-  <si>
     <t>Type</t>
   </si>
   <si>
@@ -138,6 +135,9 @@
   </si>
   <si>
     <t>Workflow</t>
+  </si>
+  <si>
+    <t>URL</t>
   </si>
 </sst>
 </file>
@@ -490,24 +490,24 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -533,151 +533,151 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
         <v>6</v>
-      </c>
-      <c r="B1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
         <v>8</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
         <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RAID-563: Fix Excel empty-cell parsing and update sentinel markers
</commit_message>
<xml_diff>
--- a/raid-agency-app/public/templates/related-objects-template.xlsx
+++ b/raid-agency-app/public/templates/related-objects-template.xlsx
@@ -126,10 +126,10 @@
     <t>No more than 100 relatedObjects can be added at one time</t>
   </si>
   <si>
-    <t>Add extra rows below the headers between the rows labelled "--- Import table starts here" and "--- Import table ends here"</t>
-  </si>
-  <si>
-    <t>Do not delete the rows labelled "--- Import table starts here" and "--- Import table ends here"</t>
+    <t>Add extra rows below the headers between the rows labelled "Import table starts here" and "Import table ends here"</t>
+  </si>
+  <si>
+    <t>Do not delete the rows labelled "Import table starts here" and "Import table ends here"</t>
   </si>
   <si>
     <t>Identifier must be the full URL of one of the types supported by RAiD. For example, a DOI would look like https://doi.org/10.0001/01238</t>
@@ -141,7 +141,7 @@
     <t>--- Instructions for use end here</t>
   </si>
   <si>
-    <t>--- Import table starts here</t>
+    <t>Import table starts here</t>
   </si>
   <si>
     <t>Identifier</t>
@@ -156,7 +156,7 @@
     <t>https://doi.org/10.0001/01238</t>
   </si>
   <si>
-    <t>--- Import table ends here</t>
+    <t>Import table ends here</t>
   </si>
 </sst>
 </file>

</xml_diff>